<commit_message>
Fix diagramador: config validator, fase3 grupos, excel writer, optimization service, eventos completos
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/diagramador_optimizado/datos_salidas.xlsx
+++ b/diagramador_optimizado/datos_salidas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lanuevametropolsa-my.sharepoint.com/personal/ccantero_grupometropol_cl/Documents/Documentos/Nueva Forma de Diagramación/Diagramación Alta 07-03-2025/Aguirre Luco/Insumos Aguirre Luco/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="665" documentId="11_7E4E55BF84DCCEE3ED7FF6F99031F45BFA722949" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9690F76-BCD6-494E-953D-CCC90074E624}"/>
+  <xr:revisionPtr revIDLastSave="669" documentId="11_7E4E55BF84DCCEE3ED7FF6F99031F45BFA722949" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F4AA356-C99D-45A7-A8EA-8CF5442A6BF8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14266,19 +14266,18 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G598" xr:uid="{12354E71-0B26-4B7B-8C25-6161D4A552EF}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e13b9520-670d-482f-8816-2d26b29eb0ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="57014138-723a-4552-b1be-d16d25732a53" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14543,21 +14542,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e13b9520-670d-482f-8816-2d26b29eb0ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="57014138-723a-4552-b1be-d16d25732a53" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11902AFE-14A7-44C5-AFCF-89115E3DAD9A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF55F5BD-32ED-43C0-82B2-325DF018CAA8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e13b9520-670d-482f-8816-2d26b29eb0ad"/>
-    <ds:schemaRef ds:uri="57014138-723a-4552-b1be-d16d25732a53"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -14582,9 +14580,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF55F5BD-32ED-43C0-82B2-325DF018CAA8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11902AFE-14A7-44C5-AFCF-89115E3DAD9A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e13b9520-670d-482f-8816-2d26b29eb0ad"/>
+    <ds:schemaRef ds:uri="57014138-723a-4552-b1be-d16d25732a53"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>